<commit_message>
﻿Test-case sheet: Notes tab shortened to a 10-row summary
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/edot-test-cases.xlsx
+++ b/docs/edot-test-cases.xlsx
@@ -1345,20 +1345,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Assertion tiers</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr"/>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Manual test cases for the web (eSuite) and mobile (eWork SFA) scope. Automation, evidence and known limits: see the repository linked in B2 of the Test Cases tab.</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1368,7 +1372,7 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>Navigation / display only; asserting the page or element is visible is enough.</t>
+          <t>Navigation / display only: the page or element is visible.</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1384,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Create/edit/delete. Assert the outcome AND the data: record exists and each value equals the input; for delete the record is gone. A success toast alone is not sufficient.</t>
+          <t>Create / edit / delete: assert the outcome AND the data (record exists, each value equals the input; after a delete the record is gone). A success toast alone is not enough.</t>
         </is>
       </c>
     </row>
@@ -1392,55 +1396,67 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Assert the specific error message text, not merely that the form is still open.</t>
+          <t>Assert the specific error message, not only that the form is still open.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="9" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Test data</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>AI-generated and schema-validated, with a Faker fallback; the values actually used are attached to the Allure report. Values in this sheet show the expected shape.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Conventions</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr"/>
+          <t>Credentials</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>No passwords or API keys in this sheet or the repo; they come from environment variables.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Credentials</t>
+          <t>Cleanup</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>No passwords/API keys are stored in this sheet or the repo; they come from environment variables (.env, gitignored).</t>
+          <t>Web: WEB-12 deletes the created company as teardown, even after earlier failures. Mobile: the app cannot delete customers, so test customers are listed in the README.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Test data</t>
+          <t>Field limit</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Company/customer data is AI-generated (schema-validated) with a deterministic Faker fallback; the values used are attached to the Allure report. Values in the sheet show the expected shape.</t>
+          <t>Company Name accepts at most 30 characters (a longer name keeps Next disabled).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cleanup</t>
+          <t>Mobile company</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>WEB-12 runs as session teardown so the shared environment is not polluted even when earlier tests fail.</t>
+          <t>Runs against the brief's fallback company 5049209 (the password comes from an environment variable).</t>
         </is>
       </c>
     </row>
@@ -1452,251 +1468,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Left blank on purpose; filled after execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="9" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Open items (to confirm by exploratory pass on the live apps before scripting)</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Login messages (captured 2 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Wrong password: banner "Incorrect password (&lt;hex reference code&gt;)" - the code is dynamic. Unknown email (contains @): dialog "Email Not Registered" + "You can continue by creating new account with this email" + the email + buttons Edit and Yes, Register. Unknown username (no @): dialog "Username Not Registered" + "We could not find an account with that username. Please check your input and try again." + the value + Edit button. Empty email: Log In button disabled.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Delete dialog (captured 2 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Red Delete button on the company's Manage page opens "Confirmation Delete": "Are you agree to delete the company? Deleting the company data will affect to other related data. You will lose all data that connected to this company in this platform and your company platform. Please consider this notice before you agree to delete." with a checkbox "I understand &amp; agree to delete", Cancel and Confirm. Confirm is disabled until the checkbox is ticked. After Confirm a toast reports that the company was deleted successfully (reported by the owner as "company delete successfully"). TBC-7 (still open): the toast's exact wording and the page shown after deletion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>TBC-8 (blocked)</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Creating a user for a new company: Company User tab &gt; + Add User (General Info: Name, Username, Employee ID, Status, Email, Phone, Password; Branch tab: Add Branch lists the company's branch, e.g. Headquarter) &gt; Submit Data. On 2 Oct 2026 Submit Data hung and the API returned {"status":500,"message":"error in account center","data":null}, also after changing username, email, phone and Employee ID to unique values. Treated as an environment/product issue, not a script defect; mobile suite uses fallback company 5049209 (declared in README).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Mobile screens (captured 2 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Login: Company ID, Username, Password (eye toggle), Sign In. Wrong password: bottom-sheet dialog "Oops" / "Wrong login combination" / OK. New Customer Registration: 3 steps Basic, Locations, Documents. Basic step: Outlet Name*, Personal/Outlet Phone No* (+62), Personal/Outlet e-mail (optional), Contact Person*, then Sales Information: Channel Type* (Choose Channel) and more. Continue is disabled on the empty form.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>TBC-11 (resolved on a device, 2 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Locations step: Address Type* (Others / Delivery Address / Invoice Address), map with "Use my current location", Address*, Province*, City*, District*, Sub district*, Postal code*, Longitude/Latitude (read-only). Documents step: KTP* number + Attachment (in-app camera), optional "Add Document"; Submit enables when both are given. Submit opens an "Approval Signature" sheet (draw a signature, then Register enables), then the confirmation "Are you sure to save this customer data?" (Yes / Cancel), then "Data Saved Successfully - saved on your device, will be uploaded when an internet connection is available". The list shows each customer as a card (name, CUST-number, distance, address, customer-type chips, status); cards are not tappable, so there is no detail screen to assert on. Customers cannot be deleted from the app, so test customers stay in the shared company (named "... QA&lt;LETTERS&gt;").</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Mobile device notes</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Real phone (Realme, Android 16). Google Password Manager can slide a "Use your saved password for ework?" sheet over the login form on launch (the flow dismisses it with Later). Maestro reinstalls its helper apps on every run unless --no-reinstall-driver is passed (the phone asks for a manual install tap each time otherwise). 4 Oct 2026: the phone keyboard's autocorrect changed a word while a value was typed ("Gatot" was saved as "Gator") and made the strict MOB-04 address assertion fail. The assertion was kept strict; the flow now checks the typed value right after typing and the test data uses plain, well-known road names. MOB-03 and MOB-04 then passed together (adb over Wi-Fi). The app cannot delete customers: the development runs left test customers (CUST-00287, 00289, 00290, 00291 and "Toko Berkah Utama QABPCSG" at least) in company 5049209.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="9" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Observed on the live eSuite (read-only pass, 2 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Menu / dashboard</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Home, Companies, Settings. Dashboard shows "Welcome Back,". Companies page: My Company, Manage Company, + Add Company, tabs Single Company / Group Company / Log Activity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Wizard step 1/3</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Fields: Company Name, Email, Phone (+62 code dropdown), Industry Type, Company Type, Language, Street Address, Country, then Province, City, District, Sub District, Postal Code (read-only, auto-filled). Next disabled until valid. Banner: free trial 30 days (a new company is Active).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Wizard step 2/3</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Step 2 "Register Legal": only an optional Legal Document (+ Add Document); Back / Next. Step 3 "Create Your Branch" (optional; "If left unfilled, a default branch will be created"): Branch Name box (empty in the automated run; in an earlier manual session it was prefilled with Headquarter and offered a "Fill in with the same data from the Company records" button, so this step varies between app versions), Policy and Terms checkbox that must be ticked before Register is enabled. Register submits and returns to the Companies list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Company detail (Manage)</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Profile Account tab: Company Name, Company ID (read-only), Industry Type, Company Type, Number of Employee (default 5 - 20 Employees), Country, Province, City, District, Sub District, Postal Code, Email, Mobile Number, Telephone, Company Address (textarea); Save Changes and a red Delete button. Other tabs: Company User, User Group, Role &amp; Permission, Legal, Currency, ... Dummy company created once in the exploratory pass must be deleted by the owner.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Typing note</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>In the in-app browser the Company Name field only accepted input after being focused via script; Playwright keyboard input is expected to behave normally but this is to be confirmed in the first run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Industry Type options</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Retail, Real Estate, Nonprofit and Social Services, Manufacturing, Hospitality, Food &amp; Beverage, Finance and Banking, Transportation and Logistics, Telecommunications, Technology, Construction, Mining and Metals, Automotive, Fast Moving Customer Goods (FMCG), Entertainment and Media, Energy, Agriculture, Healthcare, Education</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Company Type options</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Importer/Exporter, Consignor/Consignee, Marketplace, Retailer, Service Aggregator, Third-Party Logistics (3PL) Provider, Holding Company, Cooperative (Co-op), Franchisee/Franchisor, Manufacturer, Principal, Agent, Dropshipper, Freight Forwarder, Distributor, Service, Service Provider</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Language / Country options</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Language: Indonesia, English. Country: Cambodia, Philippines, Malaysia, Indonesia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Locators</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>No data-testid, and inputs have no name/id (placeholders only, e.g. "Input Company Name"). Page objects use role + accessible name / placeholder; any text locator is justified in a comment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Validation</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>No inline error text seen for invalid email or empty name; Next stays disabled (negative cases assert that).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Mobile fallback company</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard lists QA Production, ID 5049209, status Active (the brief's fallback company).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
-      <c r="B32" s="9" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Rule</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Expected texts are captured verbatim from the product and are never adjusted to match a failing run.</t>
+          <t>Left blank on purpose, as the brief asks.</t>
         </is>
       </c>
     </row>

</xml_diff>